<commit_message>
feat: Enhance model validation and editing features
- Added validation for reaction and transition consistency in ModelDocument.
- Implemented a new method to validate reaction transitions in ModelWorkspaceValidator.
- Introduced context menu options for adding and removing reactions in the main UI.
- Created ModelTableEditor for managing reactions in the model table.
- Added unit tests for ModelReactionParser, ModelTableEditor, and ModelWorkspaceValidator to ensure robustness.
- Updated existing tests to cover new validation scenarios and context menu functionality.
</commit_message>
<xml_diff>
--- a/tutorial/TCA (INST-MFA)/model/metabolic_network.xlsx
+++ b/tutorial/TCA (INST-MFA)/model/metabolic_network.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="libxl" lastEdited="7" lowestEdited="7" rupBuild="4.6.0"/>
+  <workbookPr filterPrivacy="true" defaultThemeVersion="166925"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3980F3-2D42-47F1-B125-95C4DF61AB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="5" r:id="rId1"/>
@@ -15,7 +15,7 @@
     <sheet name="biomass" sheetId="1" r:id="rId5"/>
     <sheet name="position" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="132" uniqueCount="74">
   <si>
     <t>ID</t>
   </si>
@@ -291,12 +291,15 @@
   </si>
   <si>
     <t>AKG --&gt; AlphaKetoglutarate</t>
+  </si>
+  <si>
+    <t>A &lt;=&gt; A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <fonts count="4">
     <font>
       <sz val="11"/>
@@ -335,7 +338,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -343,6 +346,7 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -350,18 +354,19 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="true"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 2" xfId="1" xr:uid="{8D570718-9775-477B-8191-F64E65370BD9}"/>
+    <cellStyle name="標準 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -377,7 +382,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -528,7 +533,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -552,9 +557,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -578,7 +583,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -613,7 +618,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -631,7 +636,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -656,7 +661,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -736,209 +741,209 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A6BC537-60DB-4B7B-B1A5-24E0DE9ADD88}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A6BC537-60DB-4B7B-B1A5-24E0DE9ADD88}">
   <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.85546875" bestFit="true" customWidth="true"/>
+    <col min="2" max="2" width="21.28515625" bestFit="true" customWidth="true"/>
+    <col min="3" max="3" width="20" bestFit="true" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" bestFit="true" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+    <row r="2">
+      <c r="A2" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="0" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="D2" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>37</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="D3" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="0" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+      <c r="D4" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="0" t="s">
         <v>40</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+      <c r="D5" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>43</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+      <c r="D6" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="0" t="s">
         <v>46</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="0" t="s">
         <v>45</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
+      <c r="D8" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>49</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" t="b">
+        <v>65</v>
+      </c>
+      <c r="D9" s="0" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
+    <row r="10">
+      <c r="A10" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
+      <c r="D11" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="0" t="s">
         <v>56</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D12" t="b">
+        <v>73</v>
+      </c>
+      <c r="D12" s="0" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13">
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14">
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15">
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16">
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="3:3">
+    <row r="17">
       <c r="C17" s="1"/>
     </row>
-    <row r="18" spans="3:3">
+    <row r="18">
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="3:3">
+    <row r="19">
       <c r="C19" s="1"/>
     </row>
-    <row r="20" spans="3:3">
+    <row r="20">
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="3:3">
+    <row r="21">
       <c r="C21" s="1"/>
     </row>
   </sheetData>

</xml_diff>